<commit_message>
docs 업데이트 (2026-05-29 01:42)
</commit_message>
<xml_diff>
--- a/docs/eland_hr_faq.xlsx
+++ b/docs/eland_hr_faq.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="6" customWidth="1" style="8" min="1" max="1"/>
@@ -823,26 +823,6 @@
       <c r="D16" s="5" t="inlineStr">
         <is>
           <t>인사팀에서 발송한 사용계획서 양식에 조직명, 사번, 이름, 잔여일수, 사용예정 날짜(월/일)를 기재합니다. 작성 후 본인 서명하여 JHO 또는 부서 근태담당자에게 제출하시면 됩니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>연차/휴가</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>10년 이상 근속 시 유급휴가 일수가 궁금합니다</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>3년차부터 2년에 한번 1일씩 가산됩니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs 업데이트 (2026-05-29 01:48)
</commit_message>
<xml_diff>
--- a/docs/eland_hr_faq.xlsx
+++ b/docs/eland_hr_faq.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="6" customWidth="1" style="8" min="1" max="1"/>
@@ -823,6 +823,26 @@
       <c r="D16" s="5" t="inlineStr">
         <is>
           <t>인사팀에서 발송한 사용계획서 양식에 조직명, 사번, 이름, 잔여일수, 사용예정 날짜(월/일)를 기재합니다. 작성 후 본인 서명하여 JHO 또는 부서 근태담당자에게 제출하시면 됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>연차/휴가</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>연차유급휴가 잔여일수 조회 방법이 궁금합니다.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>포탈에서 확인 가능합니다. 혹은 010-1234-5678번으로 문의 주세요.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs 업데이트 (2026-05-29 01:52)
</commit_message>
<xml_diff>
--- a/docs/eland_hr_faq.xlsx
+++ b/docs/eland_hr_faq.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="6" customWidth="1" style="8" min="1" max="1"/>
@@ -823,26 +823,6 @@
       <c r="D16" s="5" t="inlineStr">
         <is>
           <t>인사팀에서 발송한 사용계획서 양식에 조직명, 사번, 이름, 잔여일수, 사용예정 날짜(월/일)를 기재합니다. 작성 후 본인 서명하여 JHO 또는 부서 근태담당자에게 제출하시면 됩니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>연차/휴가</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>연차유급휴가 잔여일수 조회 방법이 궁금합니다.</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>포탈에서 확인 가능합니다. 혹은 010-1234-5678번으로 문의 주세요.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs 업데이트 (2026-05-29 02:04)
</commit_message>
<xml_diff>
--- a/docs/eland_hr_faq.xlsx
+++ b/docs/eland_hr_faq.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="6" customWidth="1" style="8" min="1" max="1"/>
@@ -823,6 +823,26 @@
       <c r="D16" s="5" t="inlineStr">
         <is>
           <t>인사팀에서 발송한 사용계획서 양식에 조직명, 사번, 이름, 잔여일수, 사용예정 날짜(월/일)를 기재합니다. 작성 후 본인 서명하여 JHO 또는 부서 근태담당자에게 제출하시면 됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>연차/휴가</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>10년 근속시 연차유급휴가에 대한 포상이 있는지 궁금합니다</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>별도의 연차휴가 추가 포상은 주어지지 않지만, 대신 포상휴가가 주어집니다. 자세한 내용은 010-1234-5678로 문의주세요.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs 업데이트 (2026-05-29 20:17)
</commit_message>
<xml_diff>
--- a/docs/eland_hr_faq.xlsx
+++ b/docs/eland_hr_faq.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="6" customWidth="1" style="8" min="1" max="1"/>
@@ -843,6 +843,26 @@
       <c r="D17" t="inlineStr">
         <is>
           <t>별도의 연차휴가 추가 포상은 주어지지 않지만, 대신 포상휴가가 주어집니다. 자세한 내용은 010-1234-5678로 문의주세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>연차/휴가</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>사번 조회방법이 궁금합니다.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>포털에서 확인 가능합니다:)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs 업데이트 (2026-05-29 21:30)
</commit_message>
<xml_diff>
--- a/docs/eland_hr_faq.xlsx
+++ b/docs/eland_hr_faq.xlsx
@@ -857,12 +857,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>사번 조회방법이 궁금합니다.</t>
+          <t>부서 근태담당자님의 연락처가 궁금합니다.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>포털에서 확인 가능합니다:)</t>
+          <t>010-1234-5678입니다.</t>
         </is>
       </c>
     </row>

</xml_diff>